<commit_message>
Initialization for the scalability analysis I only show the nb of order from 1/9/24 - 1/9/25, the revenue generated and the distinction between the aq line and the core nutrywell ligne.
</commit_message>
<xml_diff>
--- a/Info_W3/NutrYWell_DATASET_W3.xlsx
+++ b/Info_W3/NutrYWell_DATASET_W3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ULB\MA2\Q2\Supply Chain Performance Analytics\Business-Case-NutryWell\Info_W3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D857DA1-69BD-4D0F-91A9-814C88790ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2D4194-917D-41B4-BBC8-72756EEFCFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="3" activeTab="4" xr2:uid="{AF2A3348-3CF8-4F20-8540-295153672AF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="3" activeTab="5" xr2:uid="{AF2A3348-3CF8-4F20-8540-295153672AF7}"/>
   </bookViews>
   <sheets>
     <sheet name="GUIDE" sheetId="7" r:id="rId1"/>
@@ -2181,21 +2181,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="38">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     </dxf>
@@ -2267,13 +2263,10 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2281,9 +2274,6 @@
           <color auto="1"/>
         </top>
       </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2429,10 +2419,17 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2440,6 +2437,9 @@
           <color auto="1"/>
         </top>
       </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2547,7 +2547,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33377E52-640A-4A80-8241-A1319CD5DE5A}" name="Table1" displayName="Table1" ref="A1:F10" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" tableBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{33377E52-640A-4A80-8241-A1319CD5DE5A}" name="Table1" displayName="Table1" ref="A1:F10" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
   <autoFilter ref="A1:F10" xr:uid="{33377E52-640A-4A80-8241-A1319CD5DE5A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{F73FBEBD-5428-4AD8-A56D-79E02A5DB96C}" name="Site Code"/>
@@ -2562,19 +2562,19 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{22F8D7A5-2DEA-4B93-9971-3DBB258E4ABE}" name="Table2" displayName="Table2" ref="A1:K4" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{22F8D7A5-2DEA-4B93-9971-3DBB258E4ABE}" name="Table2" displayName="Table2" ref="A1:K4" totalsRowShown="0" headerRowDxfId="26" dataDxfId="24" headerRowBorderDxfId="25" tableBorderDxfId="23">
   <autoFilter ref="A1:K4" xr:uid="{22F8D7A5-2DEA-4B93-9971-3DBB258E4ABE}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{4A92C7EE-DB90-4D27-B3E3-9B45DEF0A476}" name="SKU"/>
     <tableColumn id="2" xr3:uid="{9060CAF8-E340-4D28-930D-5274D8F70297}" name="Product Name"/>
-    <tableColumn id="3" xr3:uid="{1669914F-809B-4898-BE69-0DAA483AB37E}" name="Launch Date" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{1669914F-809B-4898-BE69-0DAA483AB37E}" name="Launch Date" dataDxfId="22"/>
     <tableColumn id="4" xr3:uid="{FACB27F2-EFDB-4522-8EAC-C91D8290E1D2}" name="Sub-Category"/>
-    <tableColumn id="5" xr3:uid="{77CFED15-0B93-4545-AEAE-365B08C3F307}" name="Selling Price EUR" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{91265341-A882-4E94-B1DE-DA77C35B6FA3}" name="Gross Margin %" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{24A04D4D-7886-44A3-9D7F-D8A875BB7D6D}" name="Seasonality" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{6D8EE34C-4940-4E82-B83B-EA483F1DDDD9}" name="Planned Volume (Units/Month)" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{77CFED15-0B93-4545-AEAE-365B08C3F307}" name="Selling Price EUR" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{91265341-A882-4E94-B1DE-DA77C35B6FA3}" name="Gross Margin %" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{24A04D4D-7886-44A3-9D7F-D8A875BB7D6D}" name="Seasonality" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{6D8EE34C-4940-4E82-B83B-EA483F1DDDD9}" name="Planned Volume (Units/Month)" dataDxfId="18"/>
     <tableColumn id="9" xr3:uid="{ADEFBB3B-6388-4492-9B66-751F02A55FBF}" name="Uncertainty Level"/>
-    <tableColumn id="10" xr3:uid="{2F7824DE-3F9F-4027-92D7-7941E3DD26A5}" name="Included in Orders Dataset" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{2F7824DE-3F9F-4027-92D7-7941E3DD26A5}" name="Included in Orders Dataset" dataDxfId="17"/>
     <tableColumn id="11" xr3:uid="{5BFCBF27-791E-47FE-B15E-D5C107B62108}" name="Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2582,7 +2582,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{044A4F28-FD8E-4285-8781-BDE429E4B4BF}" name="Table3" displayName="Table3" ref="A1:S9" totalsRowShown="0" headerRowDxfId="37" headerRowBorderDxfId="36" tableBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{044A4F28-FD8E-4285-8781-BDE429E4B4BF}" name="Table3" displayName="Table3" ref="A1:S9" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A1:S9" xr:uid="{044A4F28-FD8E-4285-8781-BDE429E4B4BF}"/>
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{6AF2F8DF-1CD5-4C11-BA2F-67F653071559}" name="SKU"/>
@@ -2594,12 +2594,12 @@
     <tableColumn id="7" xr3:uid="{F7BD1286-382B-4D87-B6B6-6FB90C1D035A}" name="Shelf Life (months)"/>
     <tableColumn id="8" xr3:uid="{43F8A532-2AF0-4D6B-8F33-87370E1498B9}" name="Selling Price EUR"/>
     <tableColumn id="9" xr3:uid="{333E642F-99FF-4CB7-A491-C1FD18F94E9A}" name="Gross Margin %"/>
-    <tableColumn id="10" xr3:uid="{457BB6AF-5331-4DA3-BD14-5305641EBDB9}" name="Launch Date" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{457BB6AF-5331-4DA3-BD14-5305641EBDB9}" name="Launch Date" dataDxfId="13"/>
     <tableColumn id="11" xr3:uid="{8F18D877-48F7-4B7A-B2F1-9DA8CD658234}" name="Seasonality"/>
     <tableColumn id="12" xr3:uid="{EC7BE6D8-2613-4682-9FDC-33EC04E2FA51}" name="Standard Cost EUR"/>
     <tableColumn id="13" xr3:uid="{A85859CE-073C-484F-AD69-51F80C534631}" name="Primary Plant"/>
     <tableColumn id="14" xr3:uid="{50F364C1-CF79-40A2-A67E-AF781CAD2862}" name="Primary DC"/>
-    <tableColumn id="15" xr3:uid="{DA86CE91-6D9A-459C-AC33-853268F9D6D5}" name="Commercial Start Date" dataDxfId="33"/>
+    <tableColumn id="15" xr3:uid="{DA86CE91-6D9A-459C-AC33-853268F9D6D5}" name="Commercial Start Date" dataDxfId="12"/>
     <tableColumn id="16" xr3:uid="{477D57E6-900E-46E8-AF7E-61AB9BCC3034}" name="Included in Orders Dataset"/>
     <tableColumn id="17" xr3:uid="{9AA0E1EA-88DC-4692-B51D-48DCF4045C79}" name="Notes"/>
     <tableColumn id="18" xr3:uid="{536D19D4-28A6-4ACA-90C3-D132817E154E}" name="Forecast Monthly Demand (units)"/>
@@ -2610,17 +2610,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2EEDAB05-8C82-44D7-ACAB-A3DB37D5C0A4}" name="Table4" displayName="Table4" ref="A1:H18" totalsRowShown="0" headerRowDxfId="19" dataDxfId="17" headerRowBorderDxfId="18" tableBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{2EEDAB05-8C82-44D7-ACAB-A3DB37D5C0A4}" name="Table4" displayName="Table4" ref="A1:H18" totalsRowShown="0" headerRowDxfId="37" dataDxfId="35" headerRowBorderDxfId="36" tableBorderDxfId="34">
   <autoFilter ref="A1:H18" xr:uid="{2EEDAB05-8C82-44D7-ACAB-A3DB37D5C0A4}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{C400AC16-06F3-40CD-8CD0-8199522E3567}" name="SKU"/>
     <tableColumn id="2" xr3:uid="{8745CEAB-ECBB-45FD-B722-F2A10C3D1B92}" name="Product Name"/>
     <tableColumn id="3" xr3:uid="{0E4579E5-FB29-42B0-85E6-AEC31B8A6E84}" name="Primary Production Site"/>
     <tableColumn id="4" xr3:uid="{C8DE4DB7-792C-4C24-81A0-8483C84B7E7C}" name="Primary DC"/>
-    <tableColumn id="5" xr3:uid="{BC9C5850-1157-4602-A654-9214E1B7E529}" name="Production Lead Time (days)" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{E302385E-AC2D-4E25-9495-225B1E51368E}" name="QA Release Lead Time (days)" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{E097725B-E503-4893-A34D-8C4AE99896E8}" name="Plant → DC Shipping Lead Time (days)" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{AE6C2FA0-D663-4BC9-A18F-4FFDAF4B25F8}" name="Total time for production and delivery" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{BC9C5850-1157-4602-A654-9214E1B7E529}" name="Production Lead Time (days)" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{E302385E-AC2D-4E25-9495-225B1E51368E}" name="QA Release Lead Time (days)" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{E097725B-E503-4893-A34D-8C4AE99896E8}" name="Plant → DC Shipping Lead Time (days)" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{AE6C2FA0-D663-4BC9-A18F-4FFDAF4B25F8}" name="Total time for production and delivery" dataDxfId="30">
       <calculatedColumnFormula>SUM(Table4[[#This Row],[Production Lead Time (days)]:[Plant → DC Shipping Lead Time (days)]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2629,20 +2629,23 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C7345939-7FAB-4ADA-9481-68FE8BE0F40E}" name="Table5" displayName="Table5" ref="A1:K460" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C7345939-7FAB-4ADA-9481-68FE8BE0F40E}" name="Table5" displayName="Table5" ref="A1:K460" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
   <autoFilter ref="A1:K460" xr:uid="{C7345939-7FAB-4ADA-9481-68FE8BE0F40E}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K460">
+    <sortCondition ref="B1:B460"/>
+  </sortState>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{DD590433-1C54-46AE-8219-18A1231B0B39}" name="PO ID"/>
-    <tableColumn id="2" xr3:uid="{7E126EF3-1DF7-43B1-B8F1-791ED9A07343}" name="PO Date" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{7E126EF3-1DF7-43B1-B8F1-791ED9A07343}" name="PO Date" dataDxfId="7"/>
     <tableColumn id="3" xr3:uid="{697097E2-39D6-4606-90F2-96D8E240B847}" name="Month"/>
     <tableColumn id="4" xr3:uid="{1AE665F1-7853-4DA8-832F-D1AE2A3E409E}" name="SKU"/>
-    <tableColumn id="5" xr3:uid="{C5E4B1C4-14AC-4FBE-B284-8CCCDA8D6102}" name="Purchase Multiple (units)" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{E1BDCE76-D698-495A-BA8C-958E18EB7A61}" name="Quantity Purchased (units)" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{4EA2E67A-A672-4BD1-9952-04B18A8F1068}" name="Unit Cost EUR" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{E4FA2456-CB81-4BD0-810E-713FBB191A21}" name="Total Cost EUR" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{76D6985B-9241-493C-9DF9-167597AA105A}" name="Production Site" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{1073817C-B1CC-49D8-A60E-37F865BF321F}" name="Destination DC" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{D3F5AEB1-51C4-4486-9AD3-1623B145DAE3}" name="Goods Receipt Date" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C5E4B1C4-14AC-4FBE-B284-8CCCDA8D6102}" name="Purchase Multiple (units)" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{E1BDCE76-D698-495A-BA8C-958E18EB7A61}" name="Quantity Purchased (units)" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{4EA2E67A-A672-4BD1-9952-04B18A8F1068}" name="Unit Cost EUR" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{E4FA2456-CB81-4BD0-810E-713FBB191A21}" name="Total Cost EUR" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{76D6985B-9241-493C-9DF9-167597AA105A}" name="Production Site" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{1073817C-B1CC-49D8-A60E-37F865BF321F}" name="Destination DC" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{D3F5AEB1-51C4-4486-9AD3-1623B145DAE3}" name="Goods Receipt Date" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2938,14 +2941,14 @@
   <sheetData>
     <row r="1" spans="2:29" ht="53.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:29" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="16" t="s">
         <v>653</v>
       </c>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
     </row>
     <row r="3" spans="2:29" ht="17.5" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
@@ -3108,11 +3111,11 @@
       <c r="AC9" s="14"/>
     </row>
     <row r="10" spans="2:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
@@ -3239,11 +3242,11 @@
       <c r="AC16" s="14"/>
     </row>
     <row r="17" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
     </row>
     <row r="18" spans="2:29" x14ac:dyDescent="0.35">
       <c r="B18" s="13" t="s">
@@ -3347,11 +3350,11 @@
       <c r="AC23" s="14"/>
     </row>
     <row r="24" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
     </row>
     <row r="25" spans="2:29" x14ac:dyDescent="0.35">
       <c r="B25" s="13" t="s">
@@ -3453,11 +3456,11 @@
       <c r="AC30" s="14"/>
     </row>
     <row r="31" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
     </row>
     <row r="32" spans="2:29" x14ac:dyDescent="0.35">
       <c r="B32" s="13" t="s">
@@ -3557,11 +3560,11 @@
       <c r="AC37" s="14"/>
     </row>
     <row r="38" spans="2:29" x14ac:dyDescent="0.35">
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
     </row>
     <row r="39" spans="2:29" x14ac:dyDescent="0.35">
       <c r="B39" s="13" t="s">
@@ -3743,6 +3746,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B11:Y11"/>
+    <mergeCell ref="B4:AC4"/>
+    <mergeCell ref="B6:AC6"/>
+    <mergeCell ref="B8:AC9"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:Y39"/>
     <mergeCell ref="B15:AC16"/>
     <mergeCell ref="B17:D17"/>
@@ -3755,12 +3764,6 @@
     <mergeCell ref="B32:Y32"/>
     <mergeCell ref="B36:AC37"/>
     <mergeCell ref="B38:D38"/>
-    <mergeCell ref="B11:Y11"/>
-    <mergeCell ref="B4:AC4"/>
-    <mergeCell ref="B6:AC6"/>
-    <mergeCell ref="B8:AC9"/>
-    <mergeCell ref="H2:M2"/>
-    <mergeCell ref="B10:D10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -21492,18 +21495,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21525,18 +21528,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E25E24DF-0B51-4F57-95FD-7BE4307E4D03}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C80B32-6E14-4FEE-BB9F-112939B1E9EE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E25E24DF-0B51-4F57-95FD-7BE4307E4D03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>